<commit_message>
Fig.6/7 irregular mix: dashed switch lines at every workload change (PNG) and named vertical-line series per switch in the Excel charts; legend below
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/data/fig6_mixT.xlsx
+++ b/figs/data/fig6_mixT.xlsx
@@ -322,6 +322,294 @@
           </yVal>
           <smooth val="0"/>
         </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!Y1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$X$2:$X$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$Y$2:$Y$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AA1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$Z$2:$Z$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AA$2:$AA$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AC1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AB$2:$AB$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AC$2:$AC$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AE1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AD$2:$AD$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AE$2:$AE$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AG1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AF$2:$AF$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AG$2:$AG$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="9"/>
+          <order val="9"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AI1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AH$2:$AH$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AI$2:$AI$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="10"/>
+          <order val="10"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AK1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AJ$2:$AJ$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AK$2:$AK$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="11"/>
+          <order val="11"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AM1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AL$2:$AL$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AM$2:$AM$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
         <axId val="10"/>
         <axId val="20"/>
       </scatterChart>
@@ -455,6 +743,294 @@
           <yVal>
             <numRef>
               <f>'그림7 불규칙 혼합 10시간'!$J$2:$J$54</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!Y1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$X$2:$X$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$Y$2:$Y$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AA1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$Z$2:$Z$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AA$2:$AA$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AC1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AB$2:$AB$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AC$2:$AC$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AE1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AD$2:$AD$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AE$2:$AE$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AG1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AF$2:$AF$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AG$2:$AG$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AI1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AH$2:$AH$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AI$2:$AI$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AK1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AJ$2:$AJ$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AK$2:$AK$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AM1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AL$2:$AL$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AM$2:$AM$3</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -596,6 +1172,294 @@
           </yVal>
           <smooth val="0"/>
         </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!Y1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$X$2:$X$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$Y$2:$Y$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AA1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$Z$2:$Z$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AA$2:$AA$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AC1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AB$2:$AB$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AC$2:$AC$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AE1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AD$2:$AD$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AE$2:$AE$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AG1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AF$2:$AF$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AG$2:$AG$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AI1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AH$2:$AH$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AI$2:$AI$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AK1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AJ$2:$AJ$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AK$2:$AK$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
+          <tx>
+            <strRef>
+              <f>'그림7 불규칙 혼합 10시간'!AM1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="5A5955"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AL$2:$AL$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 불규칙 혼합 10시간'!$AM$2:$AM$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
         <axId val="10"/>
         <axId val="20"/>
       </scatterChart>
@@ -672,7 +1536,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>22</col>
+      <col>41</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
@@ -694,7 +1558,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>22</col>
+      <col>41</col>
       <colOff>0</colOff>
       <row>22</row>
       <rowOff>0</rowOff>
@@ -716,7 +1580,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>22</col>
+      <col>41</col>
       <colOff>0</colOff>
       <row>43</row>
       <rowOff>0</rowOff>
@@ -1028,7 +1892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W61"/>
+  <dimension ref="A1:AP61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1132,6 +1996,86 @@
           <t>CAT-37 (기본값)</t>
         </is>
       </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>전환1 시간</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>→ 2. OLTP</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>전환2 시간</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>→ 3. Varmail</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>전환3 시간</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>→ 4. YCSB-A</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>전환4 시간</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>→ 5. YCSB-B</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>전환5 시간</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>→ 6. FIO-Fast</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>전환6 시간</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>→ 7. Varmail</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>전환7 시간</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>→ 8. YCSB-A</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>전환8 시간</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>→ 9. OLTP</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1198,6 +2142,54 @@
       <c r="U2" t="n">
         <v>1.027</v>
       </c>
+      <c r="X2" t="n">
+        <v>1.118</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>3.362</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>4.475</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>5.591</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>6.703</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>7.815</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>8.930999999999999</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1263,6 +2255,54 @@
       </c>
       <c r="U3" t="n">
         <v>1.179</v>
+      </c>
+      <c r="X3" t="n">
+        <v>1.118</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>60</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>60</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>3.362</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>60</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>4.475</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>60</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>5.591</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>60</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>6.703</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>60</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>7.815</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>60</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>8.930999999999999</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="4">

</xml_diff>